<commit_message>
Update Performance of models.xlsx
</commit_message>
<xml_diff>
--- a/Performance of models.xlsx
+++ b/Performance of models.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\iCloudDrive\Cand.Merc BI\Speciale\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\OneDrive\Desktop\Stock predictor project V2\Carbohydrate-Estimation-for-Diabetes-management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64233657-C805-474B-90C9-4E5F3259C53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBEEC782-E7E4-4E45-A4BF-9217D58A04EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{17860A22-7D68-4CAD-9203-492DA2544ABD}"/>
   </bookViews>
@@ -168,15 +168,6 @@
     <t>PMAE</t>
   </si>
   <si>
-    <t>Model 12 (RGB transformer + ingredient oracle)</t>
-  </si>
-  <si>
-    <t>Model 11 (RGB transformer + Mass + ingredient oracle)</t>
-  </si>
-  <si>
-    <t>Model 10 (RGB transformer + Mass oracle)</t>
-  </si>
-  <si>
     <t>Model 9 V2 (RGB + side angle image mass estimator)</t>
   </si>
   <si>
@@ -256,6 +247,15 @@
   </si>
   <si>
     <t>Model 27 RDInet carbohydrate estimator + ingredient estimator + mass estimator</t>
+  </si>
+  <si>
+    <t>Model 10 (RGB transformer + Mass ground truth)</t>
+  </si>
+  <si>
+    <t>Model 11 (RGB transformer + Mass + ingredient ground truth)</t>
+  </si>
+  <si>
+    <t>Model 12 (RGB transformer + ingredient ground truth)</t>
   </si>
 </sst>
 </file>
@@ -818,7 +818,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -967,7 +967,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>70.5732</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B22">
         <v>71.5792</v>
@@ -1140,7 +1140,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="B23">
         <v>53.767899999999997</v>
@@ -1158,7 +1158,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B24">
         <v>44.950200000000002</v>
@@ -1176,7 +1176,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B25">
         <v>48.992100000000001</v>
@@ -1194,7 +1194,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="B26">
         <v>55.998100000000001</v>
@@ -1212,7 +1212,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B27">
         <v>75.341700000000003</v>
@@ -1225,12 +1225,12 @@
         <v>8.6799596773256962</v>
       </c>
       <c r="F27" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28">
         <v>85.885499999999993</v>
@@ -1245,10 +1245,10 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D29" t="e">
         <f t="shared" ref="D29:D33" si="2">SQRT(B29)</f>
@@ -1257,7 +1257,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>206.46209999999999</v>
@@ -1272,7 +1272,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B31">
         <v>232.74950000000001</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B32">
         <v>68.819699999999997</v>
@@ -1302,22 +1302,22 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B33">
-        <v>71.837400000000002</v>
+        <v>51.511899999999997</v>
       </c>
       <c r="C33">
-        <v>5.2866</v>
+        <v>4.5335000000000001</v>
       </c>
       <c r="D33">
         <f t="shared" si="2"/>
-        <v>8.4756946617961653</v>
+        <v>7.1771791116008803</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B34">
         <v>50.892932999999999</v>
@@ -1326,7 +1326,7 @@
         <v>4.6186860000000003</v>
       </c>
       <c r="D34">
-        <f>SQRT(B34)</f>
+        <f t="shared" ref="D34:D39" si="3">SQRT(B34)</f>
         <v>7.1339283007330536</v>
       </c>
       <c r="E34">
@@ -1335,7 +1335,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B35">
         <v>55.817585000000001</v>
@@ -1344,7 +1344,7 @@
         <v>4.5983049999999999</v>
       </c>
       <c r="D35">
-        <f>SQRT(B35)</f>
+        <f t="shared" si="3"/>
         <v>7.4711167170644579</v>
       </c>
       <c r="E35">
@@ -1353,7 +1353,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B36">
         <v>53.892200000000003</v>
@@ -1362,7 +1362,7 @@
         <v>4.7191000000000001</v>
       </c>
       <c r="D36">
-        <f>SQRT(B36)</f>
+        <f t="shared" si="3"/>
         <v>7.3411307031001707</v>
       </c>
       <c r="E36">
@@ -1371,7 +1371,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B37">
         <v>55.001998999999998</v>
@@ -1380,13 +1380,13 @@
         <v>4.9486369999999997</v>
       </c>
       <c r="D37">
-        <f>SQRT(B37)</f>
+        <f t="shared" si="3"/>
         <v>7.4163332584235988</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B38">
         <v>53.029980000000002</v>
@@ -1395,13 +1395,13 @@
         <v>4.7144979999999999</v>
       </c>
       <c r="D38">
-        <f>SQRT(B38)</f>
+        <f t="shared" si="3"/>
         <v>7.2821686330378261</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B39">
         <v>58.736553000000001</v>
@@ -1410,7 +1410,7 @@
         <v>5.124676</v>
       </c>
       <c r="D39">
-        <f>SQRT(B39)</f>
+        <f t="shared" si="3"/>
         <v>7.6639776226186882</v>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1452,7 +1452,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B45">
         <v>1944.3548000000001</v>
@@ -1467,7 +1467,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -1478,12 +1478,12 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B50">
         <v>7.1410000000000001E-2</v>
@@ -1494,17 +1494,17 @@
     </row>
     <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="67" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>